<commit_message>
Reports response fast creted
</commit_message>
<xml_diff>
--- a/sales report format.xlsx
+++ b/sales report format.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\2025\Desktop\Mis Data\Reports Drishti\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\report-app\Drishti-Reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CFE4AE09-B2CE-4169-A61F-143ECD038D45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B6AB868-6F95-44B9-8D76-5D630305684C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{B453DA22-0880-431E-A378-696EADB37D37}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="11520" xr2:uid="{B453DA22-0880-431E-A378-696EADB37D37}"/>
   </bookViews>
   <sheets>
     <sheet name="Data Scrubbing" sheetId="2" r:id="rId1"/>
@@ -102,9 +102,6 @@
     <t>user Talk Time</t>
   </si>
   <si>
-    <t>to be delete</t>
-  </si>
-  <si>
     <t>Customer Hangup</t>
   </si>
   <si>
@@ -112,6 +109,9 @@
   </si>
   <si>
     <t>&lt;=5 Sec</t>
+  </si>
+  <si>
+    <t>to be exclude</t>
   </si>
 </sst>
 </file>
@@ -184,12 +184,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -527,16 +527,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F6186AA-EED9-4821-84BC-0218C4C29A0E}">
   <dimension ref="A3:E8"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -547,42 +547,42 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B6" s="2" t="s">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B6" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B7" s="4" t="s">
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B7" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="E7" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E7" s="5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2</v>
       </c>
       <c r="B8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" t="s">
         <v>22</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>23</v>
       </c>
-      <c r="D8" t="s">
-        <v>24</v>
-      </c>
-      <c r="E8" s="2"/>
+      <c r="E8" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -596,38 +596,38 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{948D8CE2-1394-40A6-95E5-1BDAACD7CA13}">
   <dimension ref="B2:K9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.85546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="16" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.77734375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="C2" s="4" t="s">
+    <row r="2" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="C2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5" t="s">
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="H2" s="5"/>
-      <c r="I2" s="5"/>
-      <c r="J2" s="5"/>
-      <c r="K2" s="5"/>
-    </row>
-    <row r="3" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+    </row>
+    <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
         <v>0</v>
       </c>
@@ -659,7 +659,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>13</v>
       </c>
@@ -679,15 +679,15 @@
       <c r="G4">
         <v>2800</v>
       </c>
-      <c r="H4" s="3">
+      <c r="H4" s="2">
         <f>D4/C4</f>
         <v>0.45</v>
       </c>
-      <c r="I4" s="3">
+      <c r="I4" s="2">
         <f>E4/C4</f>
         <v>0.375</v>
       </c>
-      <c r="J4" s="3">
+      <c r="J4" s="2">
         <f>E4/D4</f>
         <v>0.83333333333333337</v>
       </c>
@@ -696,24 +696,24 @@
         <v>1050</v>
       </c>
     </row>
-    <row r="7" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="C7" s="4" t="s">
+    <row r="7" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="C7" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5" t="s">
+      <c r="E7" s="4"/>
+      <c r="F7" s="4"/>
+      <c r="G7" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="H7" s="5"/>
-      <c r="I7" s="5"/>
-      <c r="J7" s="5"/>
-      <c r="K7" s="5"/>
-    </row>
-    <row r="8" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="H7" s="4"/>
+      <c r="I7" s="4"/>
+      <c r="J7" s="4"/>
+      <c r="K7" s="4"/>
+    </row>
+    <row r="8" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B8" s="1" t="s">
         <v>0</v>
       </c>
@@ -745,7 +745,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>14</v>
       </c>
@@ -765,15 +765,15 @@
       <c r="G9">
         <v>2800</v>
       </c>
-      <c r="H9" s="3">
+      <c r="H9" s="2">
         <f>D9/C9</f>
         <v>0.45</v>
       </c>
-      <c r="I9" s="3">
+      <c r="I9" s="2">
         <f>E9/C9</f>
         <v>0.375</v>
       </c>
-      <c r="J9" s="3">
+      <c r="J9" s="2">
         <f>E9/D9</f>
         <v>0.83333333333333337</v>
       </c>

</xml_diff>